<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.003-01 Le seau jaune de Raphaël
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parc, bac à sable</t>
+          <t>parc, bac à sable, banc, chemin vers la maison</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut faire chanter le sable dans le seau jaune. L'heure arrive. Il prend le seau. Le doudou gris et le manteau bleu sont encore au banc. Il revient les chercher. Ils rentrent avec tout.</t>
+          <t>La barrière du parc cliquette. Sur le rebord jaune, un grain de sable brille. Raphaël veut le seau plein, maintenant, à la maison. Il verse trop vite, puis court avec le seau seul : l'anse glisse. Il refuse de foncer, met le manteau, reprend le doudou. Devant la porte, le grain de sable dore sur le rebord.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau saute sur la barrière. Le sable du bac est frais. Un seau jaune attend. Un doudou gris est assis sur le banc. L'ombre de papa est longue. Raphaël, tu as vu l'oiseau ? Oui. Il saute. En ce moment, Raphaël verse le sable. Il est près de papa. Il a un manteau bleu. Le manteau est un peu ouvert. Le sable glisse. Ça fait chh. Ça fait chh, papa. Oui. Le sable chante. Le seau se remplit. Puis il se vide. Le doudou reste sur le banc. Papa s'assoit un moment. Le sable est frais, hein ? Oui. Il est frais. Raphaël verse encore un peu. Ça fait encore chh. Le seau est lisse sous ses mains. Il est jaune, papa. Oui. Tout jaune. C'est l'heure. On va rentrer à la maison. Raphaël prend le seau jaune. Il marche vers la barrière. Le seau tapote contre sa jambe. Attends, Raphaël. On reprend tes affaires avant de partir. Raphaël s'arrête. Il regarde derrière lui. Le banc n'est pas vide. Tu cherches le manteau ? Raphaël revient vers le banc. Le manteau bleu est là. Il le prend. J'ai le manteau. Bien. Et le doudou ? Raphaël cherche le doudou. Le doudou gris est là. Il le prend. J'ai le doudou. Tu as le seau aussi ? Oui. Le seau jaune. Ses affaires sont avec lui. On peut partir, maintenant. Ils marchent vers la maison. Raphaël tient le seau. Le doudou est contre lui. Le manteau est sur son bras. Tu as tout, hein ? Oui. J'ai tout. Le seau tapote contre sa jambe. Le doudou sent encore le sable. Le doudou vient avec nous ? Oui. Il vient.</t>
+          <t>La barrière du parc cliquette, sous le vent. Un carré d'ombre coupe le bac. Le sable est frais, au fond. Sur le rebord jaune, un grain de sable brille. Il est tout petit, papa. C'est un grain du bac. Le seau jaune attend près des pieds. Le bois du banc sent le soleil. Un doudou gris est assis dessus. Le manteau bleu dort à côté. L'air sent l'herbe et le sable chaud. Raphaël, tu sens le sable ? Oui, papa. Je le verse, maintenant ! Le bac est frais, hein ? Oui. Il est frais. En ce moment, Raphaël saisit le seau. Le plastique est lisse, un peu chaud. Une poignée glisse, puis une autre. Ça fait chh, contre le plastique. Ça chante, papa. Oui, le sable chante. Raphaël veut le seau plein. Je le ramène à la maison. Le seau se remplit, lourd. Il est jaune, papa. Oui, bien jaune. C'est l'heure, Raphaël. On rentre. Attends, je le remplis ! Il verse trop vite, d'un coup. Le seau penche sur le bord. Une vague de sable touche ses chaussures. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je prends le seau, et je cours ! Il marche vers la barrière. Le seau tapote contre sa jambe. Attends, Raphaël. Ton manteau est au banc. Raphaël s'arrête. Il regarde derrière lui. Le banc n'est pas vide. Je reviens après ! Il tire l'anse, d'un coup. L'anse glisse entre ses doigts. Le seau tape le bord du bac. Le grain de sable bascule, puis tient. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes le banc ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau saute sur la barrière. Le sable du bac est frais. Un seau jaune attend. Un doudou gris est assis sur le banc. L'ombre de papa est longue. Raphaël, tu as vu l'oiseau ? Oui. Il saute. En ce moment, Raphaël verse le sable. Il est près de papa. Il a un manteau bleu. Le manteau est un peu ouvert. Le sable glisse. Ça fait chh. Ça fait chh, papa. Oui. Le sable chante. Le seau se remplit. Puis il se vide. Le doudou reste sur le banc. Papa s'assoit un moment. Le sable est frais, hein ? Oui. Il est frais. Raphaël verse encore un peu. Ça fait encore chh. Le seau est lisse sous ses mains. Il est jaune, papa. Oui. Tout jaune. C'est l'heure. On va rentrer à la maison. Raphaël prend le seau jaune. Il marche vers la barrière. Le seau tapote contre sa jambe. Attends, Raphaël. On reprend tes affaires avant de partir. Raphaël s'arrête. Il regarde derrière lui. Le banc n'est pas vide. Tu cherches le manteau ? Raphaël revient vers le banc. Le manteau bleu est là. Il le prend. J'ai le manteau. Bien. Et le doudou ? Raphaël cherche le doudou. Le doudou gris est là. Il le prend. J'ai le doudou. Tu as le seau aussi ? Oui. Le seau jaune. Ses affaires sont avec lui. On peut partir, maintenant. Ils marchent vers la maison. Raphaël tient le seau. Le doudou est contre lui. Le manteau est sur son bras. Tu as tout, hein ? Oui. J'ai tout. Le seau tapote contre sa jambe. Le doudou sent encore le sable. Le doudou vient avec nous ? Oui. Il vient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La barrière du parc cliquette, sous le vent. Un carré d'ombre coupe le bac. Le sable est frais, au fond. Sur le rebord jaune, un &lt;emphasis level="moderate"&gt;grain de sable&lt;/emphasis&gt; brille. Il est tout petit, papa. C'est un grain du bac. Le seau jaune attend près des pieds. Le bois du banc sent le soleil. Un doudou gris est assis dessus. Le manteau bleu dort à côté. L'air sent l'herbe et le sable chaud. Raphaël, tu sens le sable ? Oui, papa. Je le verse, maintenant ! Le bac est frais, hein ? Oui. Il est frais. En ce moment, Raphaël saisit le seau. Le plastique est lisse, un peu chaud. Une poignée glisse, puis une autre. Ça fait chh, contre le plastique. Ça chante, papa. Oui, le sable chante. Raphaël veut le seau plein. Je le ramène à la maison. Le seau se remplit, lourd. Il est jaune, papa. Oui, bien jaune. C'est l'heure, Raphaël. On rentre. Attends, je le remplis ! Il verse trop vite, d'un coup. Le seau penche sur le bord. Une vague de sable touche ses chaussures. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je prends le seau, et je cours ! Il marche vers la barrière. Le seau tapote contre sa jambe. Attends, Raphaël. Ton manteau est au banc. Raphaël s'arrête. Il regarde derrière lui. Le banc n'est pas vide. Je reviens après ! Il tire l'anse, d'un coup. L'anse glisse entre ses doigts. Le seau tape le bord du bac. Le grain de sable bascule, puis tient. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes le banc ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sami joue au parc, près de papa. Le sable est frais. Sami a un seau jaune. Il a un manteau bleu. Il a son doudou gris. Sami verse le sable. Ça fait chh. Papa dit : c'est l'heure. On va &lt;emphasis&gt;reprendre&lt;/emphasis&gt; ses affaires avant de partir. Sami cherche le seau. Il le prend. Sami cherche le manteau. Il le prend. Sami cherche le doudou. Il le prend. Ses affaires sont dans ses mains. Papa dit : merci Sami. Ils marchent vers la maison.&lt;/slow&gt; [pause]</t>
+          <t>La barrière du parc cliquette, sous le vent. Un carré d'ombre coupe le bac. Le sable est frais, au fond. Sur le rebord jaune, un &lt;emphasis&gt;grain de sable&lt;/emphasis&gt; brille. Il est tout petit, papa. C'est un grain du bac. Le seau jaune attend près des pieds. Le bois du banc sent le soleil. Un doudou gris est assis dessus. Le manteau bleu dort à côté. L'air sent l'herbe et le sable chaud. Raphaël, tu sens le sable ? Oui, papa. Je le verse, maintenant ! Le bac est frais, hein ? Oui. Il est frais. En ce moment, Raphaël saisit le seau. Le plastique est lisse, un peu chaud. Une poignée glisse, puis une autre. Ça fait chh, contre le plastique. Ça chante, papa. Oui, le sable chante. Raphaël veut le seau plein. Je le ramène à la maison. Le seau se remplit, lourd. Il est jaune, papa. Oui, bien jaune. C'est l'heure, Raphaël. On rentre. Attends, je le remplis ! Il verse trop vite, d'un coup. Le seau penche sur le bord. Une vague de sable touche ses chaussures. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je prends le seau, et je cours ! Il marche vers la barrière. Le seau tapote contre sa jambe. Attends, Raphaël. Ton manteau est au banc. Raphaël s'arrête. Il regarde derrière lui. Le banc n'est pas vide. Je reviens après ! Il tire l'anse, d'un coup. L'anse glisse entre ses doigts. Le seau tape le bord du bac. Le grain de sable bascule, puis tient. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes le banc ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>grain de sable</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,84 +1319,74 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_seau_plein_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un oiseau saute sur la barrière.
-narrateur|Le sable du bac est frais.
-narrateur|Un seau jaune attend.
-narrateur|Un doudou gris est assis sur le banc.
-narrateur|L'ombre de papa est longue.
-papa|Raphaël, tu as vu l'oiseau ?
-enfant-m|Oui.
-enfant-m|Il saute.
-narrateur|En ce moment, Raphaël verse le sable.
-narrateur|Il est près de papa.
-narrateur|Il a un manteau bleu.
-narrateur|Le manteau est un peu ouvert.
-narrateur|Le sable glisse.
-narrateur|Ça fait chh.
-enfant-m|Ça fait chh, papa.
-papa|Oui.
-papa|Le sable chante.
-narrateur|Le seau se remplit.
-narrateur|Puis il se vide.
-narrateur|Le doudou reste sur le banc.
-narrateur|Papa s'assoit un moment.
-papa|Le sable est frais, hein ?
+          <t>narrateur|La barrière du parc cliquette, sous le vent.
+narrateur|Un carré d'ombre coupe le bac.
+narrateur|Le sable est frais, au fond.
+narrateur|Sur le rebord jaune, un grain de sable brille.
+enfant-m|Il est tout petit, papa.
+papa|C'est un grain du bac.
+narrateur|Le seau jaune attend près des pieds.
+narrateur|Le bois du banc sent le soleil.
+narrateur|Un doudou gris est assis dessus.
+narrateur|Le manteau bleu dort à côté.
+narrateur|L'air sent l'herbe et le sable chaud.
+papa|Raphaël, tu sens le sable ?
+enfant-m|Oui, papa.
+enfant-m|Je le verse, maintenant !
+papa|Le bac est frais, hein ?
 enfant-m|Oui.
 enfant-m|Il est frais.
-narrateur|Raphaël verse encore un peu.
-narrateur|Ça fait encore chh.
-narrateur|Le seau est lisse sous ses mains.
+narrateur|En ce moment, Raphaël saisit le seau.
+narrateur|Le plastique est lisse, un peu chaud.
+narrateur|Une poignée glisse, puis une autre.
+narrateur|Ça fait chh, contre le plastique.
+enfant-m|Ça chante, papa.
+papa|Oui, le sable chante.
+narrateur|Raphaël veut le seau plein.
+enfant-m|Je le ramène à la maison.
+narrateur|Le seau se remplit, lourd.
 enfant-m|Il est jaune, papa.
-papa|Oui.
-papa|Tout jaune.
-papa|C'est l'heure.
-papa|On va rentrer à la maison.
-narrateur|Raphaël prend le seau jaune.
+papa|Oui, bien jaune.
+papa|C'est l'heure, Raphaël.
+papa|On rentre.
+enfant-m|Attends, je le remplis !
+narrateur|Il verse trop vite, d'un coup.
+narrateur|Le seau penche sur le bord.
+narrateur|Une vague de sable touche ses chaussures.
+enfant-m|Oh.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Je prends le seau, et je cours !
 narrateur|Il marche vers la barrière.
 narrateur|Le seau tapote contre sa jambe.
 papa|Attends, Raphaël.
-papa|On reprend tes affaires avant de partir.
+papa|Ton manteau est au banc.
 narrateur|Raphaël s'arrête.
 narrateur|Il regarde derrière lui.
 narrateur|Le banc n'est pas vide.
-papa|Tu cherches le manteau ?
-narrateur|Raphaël revient vers le banc.
-narrateur|Le manteau bleu est là.
-narrateur|Il le prend.
-enfant-m|J'ai le manteau.
-papa|Bien.
-papa|Et le doudou ?
-narrateur|Raphaël cherche le doudou.
-narrateur|Le doudou gris est là.
-narrateur|Il le prend.
-enfant-m|J'ai le doudou.
-papa|Tu as le seau aussi ?
-enfant-m|Oui.
-enfant-m|Le seau jaune.
-narrateur|Ses affaires sont avec lui.
-papa|On peut partir, maintenant.
-narrateur|Ils marchent vers la maison.
-narrateur|Raphaël tient le seau.
-narrateur|Le doudou est contre lui.
-narrateur|Le manteau est sur son bras.
-papa|Tu as tout, hein ?
-enfant-m|Oui.
-enfant-m|J'ai tout.
-narrateur|Le seau tapote contre sa jambe.
-narrateur|Le doudou sent encore le sable.
-papa|Le doudou vient avec nous ?
-enfant-m|Oui.
-enfant-m|Il vient.</t>
+enfant-m|Je reviens après !
+narrateur|Il tire l'anse, d'un coup.
+narrateur|L'anse glisse entre ses doigts.
+narrateur|Le seau tape le bord du bac.
+narrateur|Le grain de sable bascule, puis tient.
+enfant-m|Ça ne veut pas, papa.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes le banc ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>barrière,sable</t>
         </is>
       </c>
     </row>
@@ -1423,17 +1413,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Raphaël ?</t>
+          <t>Raphaël reprend ses affaires. Que fait-il, avant de partir ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Raphaël ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Raphaël reprend ses &lt;emphasis level="moderate"&gt;affaires&lt;/emphasis&gt;. Que fait-il, avant de partir ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;&lt;emphasis&gt;avant&lt;/emphasis&gt; de partir, que fait Sami ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Raphaël reprend ses &lt;emphasis&gt;affaires&lt;/emphasis&gt;. Que fait-il, avant de partir ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1443,7 +1433,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>reprendre | ses affaires | il reprend | avant de partir</t>
+          <t>reprendre | ses affaires | il reprend | avant de partir | manteau | doudou | seau</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1496,7 +1486,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1504,10 +1494,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1522,38 +1512,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>affaires</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1562,13 +1552,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1578,12 +1568,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_reprend_manteau_doudou_seau; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, que fait Raphaël ?</t>
+          <t>narrateur|Raphaël reprend ses affaires.
+narrateur|Que fait-il, avant de partir ?</t>
         </is>
       </c>
     </row>
@@ -1610,17 +1601,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a cherché. Il a repris le seau. Il a repris le manteau. Il a repris le doudou. C'était avant de partir. Tu as repris tes affaires. Avant de partir. J'ai tout, papa. Oui.</t>
+          <t>Raphaël refuse de tirer plus fort. Il pose un genou au sable. L'anse est libre, un instant. Je le sors tout seul. Il pose le seau près du banc. Le manteau, et le doudou. Il prend les deux, d'un coup. Le manteau glisse, tombe. Le doudou roule sous le banc. Oh. Il ne reprend pas trop vite. Il écoute le parc, un instant. Sur le rebord, le grain de sable brille. Il est là. Tu mets le manteau ? Raphaël prend le manteau bleu. Une manche entre, facile. L'autre manche reste coincée, derrière. Je tire ! Il s'arrête. Raphaël refuse de foncer. Il recule le bras, lentement. La manche se libère, lisse. Merci, Raphaël. Il se baisse près du bois. Ses doigts trouvent le doudou gris. Te voilà. Il le serre contre sa joue. Tu as le seau aussi ? Oui. Le seau jaune. Ses affaires sont avec lui. On peut partir ? Oui, papa. Raphaël pose la main sur l'anse. L'anse est un peu rêche.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a cherché. Il a repris le seau. Il a repris le manteau. Il a repris le doudou. C'était avant de partir. Tu as repris tes affaires. Avant de partir. J'ai tout, papa. Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël refuse de tirer plus fort. Il pose un genou au sable. L'anse est libre, un instant. Je le sors tout seul. Il pose le seau près du banc. Le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt;, et le doudou. Il prend les deux, d'un coup. Le manteau glisse, tombe. Le doudou roule sous le banc. Oh. Il ne reprend pas trop vite. Il écoute le parc, un instant. Sur le rebord, le grain de sable brille. Il est là. Tu mets le manteau ? Raphaël prend le manteau bleu. Une manche entre, facile. L'autre manche reste coincée, derrière. Je tire ! Il s'arrête. Raphaël refuse de foncer. Il recule le bras, lentement. La manche se libère, lisse. Merci, Raphaël. Il se baisse près du bois. Ses doigts trouvent le doudou gris. Te voilà. Il le serre contre sa joue. Tu as le seau aussi ? Oui. Le seau jaune. Ses affaires sont avec lui. On peut partir ? Oui, papa. Raphaël pose la main sur l'anse. L'anse est un peu rêche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sami a cherché. Il a repris le seau. Il a repris le manteau. Il a repris le doudou. C'était &lt;emphasis&gt;avant&lt;/emphasis&gt; de partir.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël refuse de tirer plus fort. Il pose un genou au sable. L'anse est libre, un instant. Je le sors tout seul. Il pose le seau près du banc. Le &lt;emphasis&gt;manteau&lt;/emphasis&gt;, et le doudou. Il prend les deux, d'un coup. Le manteau glisse, tombe. Le doudou roule sous le banc. Oh. Il ne reprend pas trop vite. Il écoute le parc, un instant. Sur le rebord, le grain de sable brille. Il est là. Tu mets le manteau ? Raphaël prend le manteau bleu. Une manche entre, facile. L'autre manche reste coincée, derrière. Je tire ! Il s'arrête. Raphaël refuse de foncer. Il recule le bras, lentement. La manche se libère, lisse. Merci, Raphaël. Il se baisse près du bois. Ses doigts trouvent le doudou gris. Te voilà. Il le serre contre sa joue. Tu as le seau aussi ? Oui. Le seau jaune. Ses affaires sont avec lui. On peut partir ? Oui, papa. Raphaël pose la main sur l'anse. L'anse est un peu rêche. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1667,18 +1658,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1701,30 +1692,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>manteau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1733,10 +1724,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1745,24 +1736,56 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_s_habille_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël a cherché.
-narrateur|Il a repris le seau.
-narrateur|Il a repris le manteau.
-narrateur|Il a repris le doudou.
-narrateur|C'était avant de partir.
-papa|Tu as repris tes affaires.
-papa|Avant de partir.
-enfant-m|J'ai tout, papa.
-papa|Oui.</t>
+          <t>narrateur|Raphaël refuse de tirer plus fort.
+narrateur|Il pose un genou au sable.
+narrateur|L'anse est libre, un instant.
+enfant-m|Je le sors tout seul.
+narrateur|Il pose le seau près du banc.
+enfant-m|Le manteau, et le doudou.
+narrateur|Il prend les deux, d'un coup.
+narrateur|Le manteau glisse, tombe.
+narrateur|Le doudou roule sous le banc.
+enfant-m|Oh.
+narrateur|Il ne reprend pas trop vite.
+narrateur|Il écoute le parc, un instant.
+narrateur|Sur le rebord, le grain de sable brille.
+enfant-m|Il est là.
+papa|Tu mets le manteau ?
+narrateur|Raphaël prend le manteau bleu.
+narrateur|Une manche entre, facile.
+narrateur|L'autre manche reste coincée, derrière.
+enfant-m|Je tire !
+narrateur|Il s'arrête.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il recule le bras, lentement.
+narrateur|La manche se libère, lisse.
+papa|Merci, Raphaël.
+narrateur|Il se baisse près du bois.
+narrateur|Ses doigts trouvent le doudou gris.
+enfant-m|Te voilà.
+narrateur|Il le serre contre sa joue.
+papa|Tu as le seau aussi ?
+enfant-m|Oui.
+enfant-m|Le seau jaune.
+narrateur|Ses affaires sont avec lui.
+papa|On peut partir ?
+enfant-m|Oui, papa.
+narrateur|Raphaël pose la main sur l'anse.
+narrateur|L'anse est un peu rêche.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>banc,manteau</t>
         </is>
       </c>
     </row>
@@ -1789,17 +1812,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël tient le seau. Le doudou est contre lui. Je marche à côté de toi. Le sable reste au parc. Tu as les affaires avec toi ? Oui, papa. L'oiseau n'est plus sur la barrière. Le banc est vide, maintenant. Le sable reste dans le bac. On rentre à la maison. Avec mes affaires. Oui.</t>
+          <t>On prend le chemin ? Raphaël serre le manteau contre lui. Une manche est tiède. Tu as ton manteau ? Oui, papa. On ouvre la barrière. Papa ouvre la barrière. L'air sent l'herbe coupée. Le seau jaune tape contre sa hanche. On rentre avec le seau ? Oui, il est à toi. Ils marchent sur le chemin. Le doudou est contre lui. Je la vois, papa ? Bientôt. On continue. Une branche traverse, plus loin. Le chemin est un peu poudreux. Une racine ronde bloque le pas. Je saute par-dessus ! Raphaël recule d'un pas. Il refuse de foncer. Il contourne la racine, lentement. Le seau reste bien droit. Ça sent bon. Oui, très bon. Raphaël sent le sable sur sa langue.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël tient le seau. Le doudou est contre lui. Je marche à côté de toi. Le sable reste au parc. Tu as les affaires avec toi ? Oui, papa. L'oiseau n'est plus sur la barrière. Le banc est vide, maintenant. Le sable reste dans le bac. On rentre à la maison. Avec mes affaires. Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On prend le chemin ? Raphaël serre le manteau contre lui. Une manche est tiède. Tu as ton manteau ? Oui, papa. On ouvre la barrière. Papa ouvre la barrière. L'air sent l'herbe coupée. Le seau jaune tape contre sa hanche. On rentre avec le seau ? Oui, il est à toi. Ils marchent sur le chemin. Le doudou est contre lui. Je la vois, papa ? Bientôt. On continue. Une branche traverse, plus loin. Le chemin est un peu poudreux. Une &lt;emphasis level="moderate"&gt;racine&lt;/emphasis&gt; ronde bloque le pas. Je saute par-dessus ! Raphaël recule d'un pas. Il refuse de foncer. Il contourne la racine, lentement. Le seau reste bien droit. Ça sent bon. Oui, très bon. Raphaël sent le sable sur sa langue.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sami tient le seau. Le doudou est contre lui. Papa est à côté.&lt;/slow&gt; [pause]</t>
+          <t>On prend le chemin ? Raphaël serre le manteau contre lui. Une manche est tiède. Tu as ton manteau ? Oui, papa. On ouvre la barrière. Papa ouvre la barrière. L'air sent l'herbe coupée. Le seau jaune tape contre sa hanche. On rentre avec le seau ? Oui, il est à toi. Ils marchent sur le chemin. Le doudou est contre lui. Je la vois, papa ? Bientôt. On continue. Une branche traverse, plus loin. Le chemin est un peu poudreux. Une &lt;emphasis&gt;racine&lt;/emphasis&gt; ronde bloque le pas. Je saute par-dessus ! Raphaël recule d'un pas. Il refuse de foncer. Il contourne la racine, lentement. Le seau reste bien droit. Ça sent bon. Oui, très bon. Raphaël sent le sable sur sa langue. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1846,18 +1869,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1878,28 +1901,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>racine</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1908,10 +1935,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1920,23 +1947,47 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_sauter_la_racine; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël tient le seau.
+          <t>papa|On prend le chemin ?
+narrateur|Raphaël serre le manteau contre lui.
+narrateur|Une manche est tiède.
+papa|Tu as ton manteau ?
+enfant-m|Oui, papa.
+papa|On ouvre la barrière.
+narrateur|Papa ouvre la barrière.
+narrateur|L'air sent l'herbe coupée.
+narrateur|Le seau jaune tape contre sa hanche.
+enfant-m|On rentre avec le seau ?
+papa|Oui, il est à toi.
+narrateur|Ils marchent sur le chemin.
 narrateur|Le doudou est contre lui.
-papa|Je marche à côté de toi.
-narrateur|Le sable reste au parc.
-papa|Tu as les affaires avec toi ?
-enfant-m|Oui, papa.
-narrateur|L'oiseau n'est plus sur la barrière.
-narrateur|Le banc est vide, maintenant.
-narrateur|Le sable reste dans le bac.
-papa|On rentre à la maison.
-enfant-m|Avec mes affaires.
-papa|Oui.</t>
+enfant-m|Je la vois, papa ?
+papa|Bientôt.
+papa|On continue.
+narrateur|Une branche traverse, plus loin.
+narrateur|Le chemin est un peu poudreux.
+narrateur|Une racine ronde bloque le pas.
+enfant-m|Je saute par-dessus !
+narrateur|Raphaël recule d'un pas.
+narrateur|Il refuse de foncer.
+narrateur|Il contourne la racine, lentement.
+narrateur|Le seau reste bien droit.
+enfant-m|Ça sent bon.
+papa|Oui, très bon.
+narrateur|Raphaël sent le sable sur sa langue.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>chemin,pas</t>
         </is>
       </c>
     </row>
@@ -1963,17 +2014,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai repris mes affaires. Avant de partir. Bravo, Raphaël. Le seau jaune tapote tout doux.</t>
+          <t>Ils s'arrêtent devant la porte tiède. La chaleur touche les joues de Raphaël. La maison est là. Oui, tout près. Le seau jaune attend dans ses mains. Sur le rebord, un grain de sable brille. Comme sur le bac, papa ! Tu le portes, toi ? Oui, avec le doudou. Raphaël ouvre la porte, sans se presser. Il glisse le seau près du tapis. Le manteau repose sur le crochet. On le sent, papa. Tu le sens sur tes joues ? Oui, il est chaud. La porte tiède touche ses joues. Le grain de sable dore sur le rebord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai repris mes affaires. Avant de partir. Bravo, Raphaël. Le seau jaune tapote tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'arrêtent devant la porte tiède. La chaleur touche les joues de Raphaël. La maison est là. Oui, tout près. Le seau jaune attend dans ses mains. Sur le rebord, un &lt;emphasis level="moderate"&gt;grain de sable&lt;/emphasis&gt; brille. Comme sur le bac, papa ! Tu le portes, toi ? Oui, avec le doudou. Raphaël ouvre la porte, sans se presser. Il glisse le seau près du tapis. Le manteau repose sur le crochet. On le sent, papa. Tu le sens sur tes joues ? Oui, il est chaud. La porte tiède touche ses joues. Le grain de sable dore sur le rebord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'arrêtent devant la porte tiède. La chaleur touche les joues de Raphaël. La maison est là. Oui, tout près. Le seau jaune attend dans ses mains. Sur le rebord, un &lt;emphasis&gt;grain de sable&lt;/emphasis&gt; brille. Comme sur le bac, papa ! Tu le portes, toi ? Oui, avec le doudou. Raphaël ouvre la porte, sans se presser. Il glisse le seau près du tapis. Le manteau repose sur le crochet. On le sent, papa. Tu le sens sur tes joues ? Oui, il est chaud. La porte tiède touche ses joues. Le grain de sable dore sur le rebord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2020,7 +2071,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2028,7 +2079,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2040,12 +2091,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2054,17 +2105,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>grain de sable</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2073,11 +2128,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2086,27 +2141,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=le_grain_du_bac_est_sur_le_rebord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai repris mes affaires.
-enfant-m|Avant de partir.
-papa|Bravo, Raphaël.
-narrateur|Le seau jaune tapote tout doux.</t>
+          <t>narrateur|Ils s'arrêtent devant la porte tiède.
+narrateur|La chaleur touche les joues de Raphaël.
+enfant-m|La maison est là.
+papa|Oui, tout près.
+narrateur|Le seau jaune attend dans ses mains.
+narrateur|Sur le rebord, un grain de sable brille.
+enfant-m|Comme sur le bac, papa !
+papa|Tu le portes, toi ?
+enfant-m|Oui, avec le doudou.
+narrateur|Raphaël ouvre la porte, sans se presser.
+narrateur|Il glisse le seau près du tapis.
+narrateur|Le manteau repose sur le crochet.
+enfant-m|On le sent, papa.
+papa|Tu le sens sur tes joues ?
+enfant-m|Oui, il est chaud.
+narrateur|La porte tiède touche ses joues.
+narrateur|Le grain de sable dore sur le rebord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>porte,seau</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2219,6 +2296,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>